<commit_message>
Added HR cases template
</commit_message>
<xml_diff>
--- a/docs/פירוט דרישות.xlsx
+++ b/docs/פירוט דרישות.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shayturgeman/Desktop/הנדסת מערכות מידע/שנה ב/סמסטר ב/ניתוץ/פרויקט/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shayturgeman/Desktop/ADSS_Group_R/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1EDE329-B1A9-8148-9D0D-A8289CEE7538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6949A62D-AE9A-884F-962A-C58D2CF71BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="660" windowWidth="30240" windowHeight="17420" activeTab="1" xr2:uid="{70E4B8CB-B94F-4C8B-9B3A-24364EBEF7A3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" activeTab="1" xr2:uid="{70E4B8CB-B94F-4C8B-9B3A-24364EBEF7A3}"/>
   </bookViews>
   <sheets>
     <sheet name="דרישות" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="71">
   <si>
     <t>ID</t>
   </si>
@@ -223,6 +223,33 @@
   </si>
   <si>
     <t>האם שכר העובדים הוא שעתי או גלובלי?</t>
+  </si>
+  <si>
+    <t>כן</t>
+  </si>
+  <si>
+    <t>כן, קיימת אופציה כזו</t>
+  </si>
+  <si>
+    <t>העובדים יתחברו למערכת על ידי שם משתמש וסיסמא</t>
+  </si>
+  <si>
+    <t>לא</t>
+  </si>
+  <si>
+    <t>להחלטת מנהל כוח האדם</t>
+  </si>
+  <si>
+    <t>לעובדים ולמנהל כוח האדם</t>
+  </si>
+  <si>
+    <t>שעתי</t>
+  </si>
+  <si>
+    <t>יום</t>
+  </si>
+  <si>
+    <t>לפי דרישת מנהל כוח אדם</t>
   </si>
 </sst>
 </file>
@@ -1373,14 +1400,16 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="82" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="62" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="9"/>
+      <c r="C2" s="9" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="3" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
@@ -1389,7 +1418,9 @@
       <c r="B3" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="11"/>
+      <c r="C3" s="11" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="4" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
@@ -1407,7 +1438,9 @@
       <c r="B5" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="11"/>
+      <c r="C5" s="11" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="6" spans="1:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
@@ -1416,7 +1449,9 @@
       <c r="B6" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="9"/>
+      <c r="C6" s="9" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="7" spans="1:3" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
@@ -1425,7 +1460,9 @@
       <c r="B7" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="11"/>
+      <c r="C7" s="11" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="8" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -1434,7 +1471,9 @@
       <c r="B8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="9"/>
+      <c r="C8" s="9" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="9" spans="1:3" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
@@ -1443,7 +1482,9 @@
       <c r="B9" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="11"/>
+      <c r="C9" s="11" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="10" spans="1:3" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
@@ -1452,7 +1493,9 @@
       <c r="B10" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="9"/>
+      <c r="C10" s="9" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="11" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
@@ -1461,7 +1504,9 @@
       <c r="B11" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="11"/>
+      <c r="C11" s="11" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="12" spans="1:3" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
@@ -1470,7 +1515,9 @@
       <c r="B12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="9"/>
+      <c r="C12" s="9" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="13" spans="1:3" ht="47" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
@@ -1479,7 +1526,9 @@
       <c r="B13" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="11"/>
+      <c r="C13" s="11" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="14" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
@@ -1488,7 +1537,9 @@
       <c r="B14" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="9"/>
+      <c r="C14" s="9" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="15" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
@@ -1497,7 +1548,9 @@
       <c r="B15" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="11"/>
+      <c r="C15" s="11" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="16" spans="1:3" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
@@ -1506,7 +1559,9 @@
       <c r="B16" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="9"/>
+      <c r="C16" s="9" t="s">
+        <v>68</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Editing last changes for the HR menu
</commit_message>
<xml_diff>
--- a/docs/פירוט דרישות.xlsx
+++ b/docs/פירוט דרישות.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shayturgeman/Desktop/ADSS_Group_R/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6949A62D-AE9A-884F-962A-C58D2CF71BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341C7CD9-BE78-FF44-8CD5-2708E7C84BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" activeTab="1" xr2:uid="{70E4B8CB-B94F-4C8B-9B3A-24364EBEF7A3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17540" activeTab="1" xr2:uid="{70E4B8CB-B94F-4C8B-9B3A-24364EBEF7A3}"/>
   </bookViews>
   <sheets>
     <sheet name="דרישות" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="72">
   <si>
     <t>ID</t>
   </si>
@@ -150,18 +150,12 @@
     <t>חוסר בתפקיד במשמרת</t>
   </si>
   <si>
-    <t>מה קורה כאשר אין עובד מוסמך לתפקיד הדרוש במשמרת?</t>
-  </si>
-  <si>
     <t>עדכון לוח המשמרות</t>
   </si>
   <si>
     <t>האם ניתן לעדכן ולשנות את לוח המשמרות אחרי פרסום?</t>
   </si>
   <si>
-    <t>חלקוה שווה של משמרות</t>
-  </si>
-  <si>
     <t>האם צריכה להיות חלוקה שווה של משמרות בין העובדים השונים?</t>
   </si>
   <si>
@@ -240,9 +234,6 @@
     <t>להחלטת מנהל כוח האדם</t>
   </si>
   <si>
-    <t>לעובדים ולמנהל כוח האדם</t>
-  </si>
-  <si>
     <t>שעתי</t>
   </si>
   <si>
@@ -250,6 +241,18 @@
   </si>
   <si>
     <t>לפי דרישת מנהל כוח אדם</t>
+  </si>
+  <si>
+    <t>האם ניתן לפרסם משמרת גם כאשר יש חוסר בתפקיד?</t>
+  </si>
+  <si>
+    <t>לא, המערכת מחייבת את כל התפקידים להיות מאוישים לפני פרסום המשמרות לשבוע הבא</t>
+  </si>
+  <si>
+    <t>חלוקה שווה של משמרות</t>
+  </si>
+  <si>
+    <t>לעובדים (כולל פרטים אישיים) ולמנהל כוח אדם (לא כולל פרטים אישיים)</t>
   </si>
 </sst>
 </file>
@@ -394,7 +397,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -431,6 +434,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1382,7 +1388,7 @@
   <cols>
     <col min="1" max="1" width="39.83203125" customWidth="1"/>
     <col min="2" max="2" width="109.5" customWidth="1"/>
-    <col min="3" max="3" width="54.83203125" customWidth="1"/>
+    <col min="3" max="3" width="71" customWidth="1"/>
     <col min="4" max="4" width="12.33203125" customWidth="1"/>
     <col min="5" max="5" width="13.5" customWidth="1"/>
     <col min="6" max="6" width="16.1640625" customWidth="1"/>
@@ -1408,7 +1414,7 @@
         <v>33</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.2">
@@ -1419,7 +1425,7 @@
         <v>35</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -1427,140 +1433,142 @@
         <v>36</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="9"/>
+        <v>68</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>39</v>
-      </c>
       <c r="C5" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="53" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="47" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>67</v>
+        <v>55</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Editing the excel file
</commit_message>
<xml_diff>
--- a/docs/פירוט דרישות.xlsx
+++ b/docs/פירוט דרישות.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shayturgeman/Desktop/ADSS_Group_R/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341C7CD9-BE78-FF44-8CD5-2708E7C84BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA78B9B-EB88-764F-83C8-950D46765F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17540" activeTab="1" xr2:uid="{70E4B8CB-B94F-4C8B-9B3A-24364EBEF7A3}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="71">
   <si>
     <t>ID</t>
   </si>
@@ -235,9 +235,6 @@
   </si>
   <si>
     <t>שעתי</t>
-  </si>
-  <si>
-    <t>יום</t>
   </si>
   <si>
     <t>לפי דרישת מנהל כוח אדם</t>
@@ -1433,10 +1430,10 @@
         <v>36</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>68</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
@@ -1452,7 +1449,7 @@
     </row>
     <row r="6" spans="1:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>39</v>
@@ -1535,7 +1532,7 @@
         <v>53</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1546,7 +1543,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Changes that added after bukding the nock files
</commit_message>
<xml_diff>
--- a/docs/פירוט דרישות.xlsx
+++ b/docs/פירוט דרישות.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shayturgeman/Desktop/ADSS_Group_R/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shayturgeman/Desktop/הנדסת מערכות מידע/שנה ב/סמסטר ב/ניתוץ/ADSS_Group_R/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA78B9B-EB88-764F-83C8-950D46765F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6691ACB7-A2CA-2343-AB4E-E7D360873268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17540" activeTab="1" xr2:uid="{70E4B8CB-B94F-4C8B-9B3A-24364EBEF7A3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" activeTab="1" xr2:uid="{70E4B8CB-B94F-4C8B-9B3A-24364EBEF7A3}"/>
   </bookViews>
   <sheets>
     <sheet name="דרישות" sheetId="1" r:id="rId1"/>

</xml_diff>